<commit_message>
Add silent anomalies to the generator (10% by default)
A tenth of the injected anomalies now carry no red flag: an unusual amount
with cents on a common account, on a working day that isn't a holiday,
with an ordinary description and a different approver. The recall ceiling
is then below 1, as on real ledgers. Fixtures rebuilt from the new ledger.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/idea_exports/Account Summary.xlsx
+++ b/fixtures/idea_exports/Account Summary.xlsx
@@ -455,7 +455,7 @@
         <v>3254</v>
       </c>
       <c r="C2" t="n">
-        <v>16210109.08</v>
+        <v>16157487.59</v>
       </c>
     </row>
     <row r="3">
@@ -465,10 +465,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3194</v>
+        <v>3192</v>
       </c>
       <c r="C3" t="n">
-        <v>14695780.99</v>
+        <v>14673618.06</v>
       </c>
     </row>
     <row r="4">
@@ -478,10 +478,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4464</v>
+        <v>4463</v>
       </c>
       <c r="C4" t="n">
-        <v>20899091.39</v>
+        <v>21024242.89</v>
       </c>
     </row>
     <row r="5">
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2049</v>
+        <v>2045</v>
       </c>
       <c r="C5" t="n">
-        <v>9453444.24</v>
+        <v>9253224.02</v>
       </c>
     </row>
     <row r="6">
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="C6" t="n">
-        <v>2895630.09</v>
+        <v>2717927.06</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         <v>1552</v>
       </c>
       <c r="C7" t="n">
-        <v>7253842.98</v>
+        <v>7084085.63</v>
       </c>
     </row>
     <row r="8">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="C8" t="n">
-        <v>3170921.48</v>
+        <v>3557222.08</v>
       </c>
     </row>
     <row r="9">
@@ -543,296 +543,296 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2385</v>
+        <v>2393</v>
       </c>
       <c r="C9" t="n">
-        <v>11149352.93</v>
+        <v>11230968.71</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Suspense Account 1</t>
+          <t>Suspense Account 10</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>83264.84</v>
+        <v>10999</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Suspense Account 13</t>
+          <t>Suspense Account 11</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>10999</v>
+        <v>23911.08</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Suspense Account 14</t>
+          <t>Suspense Account 12</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2</v>
       </c>
       <c r="C12" t="n">
-        <v>140000</v>
+        <v>103839.53</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Suspense Account 16</t>
+          <t>Suspense Account 13</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>33584.27</v>
+        <v>133999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Suspense Account 17</t>
+          <t>Suspense Account 15</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>48764.52</v>
+        <v>26999</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Suspense Account 18</t>
+          <t>Suspense Account 16</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>14401.63</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Suspense Account 2</t>
+          <t>Suspense Account 17</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>45999</v>
+        <v>31999</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Suspense Account 21</t>
+          <t>Suspense Account 19</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>150000</v>
+        <v>82228.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Suspense Account 24</t>
+          <t>Suspense Account 20</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>30000</v>
+        <v>48455.75</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Suspense Account 25</t>
+          <t>Suspense Account 21</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>130000</v>
+        <v>13999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Suspense Account 26</t>
+          <t>Suspense Account 22</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="n">
-        <v>44706.74</v>
+        <v>76684.47</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Suspense Account 27</t>
+          <t>Suspense Account 24</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>108280.8</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Suspense Account 28</t>
+          <t>Suspense Account 25</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>23999</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Suspense Account 29</t>
+          <t>Suspense Account 26</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>22999</v>
+        <v>59415.07</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Suspense Account 3</t>
+          <t>Suspense Account 28</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" t="n">
-        <v>103998</v>
+        <v>21656.16</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Suspense Account 30</t>
+          <t>Suspense Account 29</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>1</v>
       </c>
       <c r="C25" t="n">
-        <v>30000</v>
+        <v>22999</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Suspense Account 31</t>
+          <t>Suspense Account 30</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>10000</v>
+        <v>46999</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Suspense Account 33</t>
+          <t>Suspense Account 31</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>54999</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Suspense Account 36</t>
+          <t>Suspense Account 32</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>170000</v>
+        <v>11999</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Suspense Account 37</t>
+          <t>Suspense Account 34</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>54999</v>
+        <v>27999</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Suspense Account 39</t>
+          <t>Suspense Account 37</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>74999</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Suspense Account 4</t>
+          <t>Suspense Account 38</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>50000</v>
+        <v>27999</v>
       </c>
     </row>
     <row r="32">
@@ -845,7 +845,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="33">
@@ -858,7 +858,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="n">
-        <v>48999</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="34">
@@ -871,111 +871,111 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>19362.98</v>
+        <v>70999</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Suspense Account 43</t>
+          <t>Suspense Account 44</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>60000</v>
+        <v>94223.39999999999</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Suspense Account 44</t>
+          <t>Suspense Account 45</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="n">
-        <v>32940.21</v>
+        <v>75370.53</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Suspense Account 45</t>
+          <t>Suspense Account 46</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" t="n">
-        <v>63999</v>
+        <v>56490.81</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Suspense Account 48</t>
+          <t>Suspense Account 47</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>77999</v>
+        <v>29565.46</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Suspense Account 5</t>
+          <t>Suspense Account 48</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>71470.53999999999</v>
+        <v>26875.75</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Suspense Account 6</t>
+          <t>Suspense Account 49</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="n">
-        <v>25284.89</v>
+        <v>102999</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Suspense Account 7</t>
+          <t>Suspense Account 8</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>41049.01</v>
+        <v>63999</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Suspense Account 8</t>
+          <t>Suspense Account 9</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>160000</v>
+        <v>87999</v>
       </c>
     </row>
     <row r="43">
@@ -985,10 +985,10 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C43" t="n">
-        <v>3258851.62</v>
+        <v>3232850.62</v>
       </c>
     </row>
     <row r="44">
@@ -998,10 +998,10 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="C44" t="n">
-        <v>3932159.82</v>
+        <v>3891392.46</v>
       </c>
     </row>
     <row r="45">
@@ -1014,7 +1014,7 @@
         <v>365</v>
       </c>
       <c r="C45" t="n">
-        <v>1758205.34</v>
+        <v>1666860.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>